<commit_message>
feat(eit): update synthesis workstation and AGV integration
Align the EIT workstation registry, deck resources, and AGV transfer flow so remote arm access and frontend material synchronization behave consistently during tray handling.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/unilabos/devices/eit_synthesis_station/sheet/batch_in_tray.xlsx
+++ b/unilabos/devices/eit_synthesis_station/sheet/batch_in_tray.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Lab-OS\unilabos\devices\eit_synthesis_station\sheet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fish/Documents/GitHub/Uni-Lab-OS/unilabos/devices/eit_synthesis_station/sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D82356-8247-4779-89F3-7151EAAC8C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03FD323-E414-0944-8B75-897C381F7128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="batch_in_tray" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>position</t>
   </si>
@@ -32,6 +32,36 @@
     <t>tray_type</t>
   </si>
   <si>
+    <t>content</t>
+  </si>
+  <si>
+    <t>shelf_position</t>
+  </si>
+  <si>
+    <t>storage</t>
+  </si>
+  <si>
+    <t>TB-2-1</t>
+  </si>
+  <si>
+    <t>30 mL粉桶托盘(201000600)</t>
+  </si>
+  <si>
+    <t>3-1</t>
+  </si>
+  <si>
+    <t>对二甲胺基苯甲醛|3-2A;4-3;3,5-二甲氧基苯甲醛|4-3</t>
+  </si>
+  <si>
+    <t>TB-2-2</t>
+  </si>
+  <si>
+    <t>3-2</t>
+  </si>
+  <si>
+    <t>对苯基苯甲醛|4-3</t>
+  </si>
+  <si>
     <t>2 mL反应试管托盘(201000726) [1-24]</t>
   </si>
   <si>
@@ -71,11 +101,11 @@
     <t>125 mL试剂瓶托盘(220000023) [A1-A2]</t>
   </si>
   <si>
-    <t>content(耗材填数量; 物质填: A1|名称|2mL; B2|名称|5mg)</t>
+    <t>A1|对二甲胺基苯甲醛|2000mg;B1|3,5-二甲氧基苯甲醛|2000mg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>TB-2-1</t>
+    <t>A1|对苯基苯甲醛|2000mg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -83,7 +113,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,7 +137,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -115,12 +145,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -423,118 +475,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="23.1796875" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="80" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="125.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" ht="15">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="31.5" customHeight="1">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>24</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="39.5" customHeight="1">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="79" customHeight="1">
+      <c r="C4" s="3"/>
+      <c r="D4"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="D5"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="D6"/>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="D7"/>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="D8"/>
+      <c r="E8" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="A2:A101" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="A2:A91" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"TB-1-1,TB-1-2,TB-1-3,TB-1-4,TB-2-1,TB-2-2,TB-2-3,TB-2-4,W-1-1,W-1-2,W-1-3,W-1-4,W-1-5,W-1-6,W-1-7,W-1-8"</formula1>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" sqref="B2:B101" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" showInputMessage="1" sqref="B2:B91" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>tray_type_options</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="64" orientation="landscape" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A13"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>